<commit_message>
refactor: update login negative test case title to specify username and password fields in Excel
</commit_message>
<xml_diff>
--- a/testcase/tc_orangehrm.xlsx
+++ b/testcase/tc_orangehrm.xlsx
@@ -635,7 +635,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Melakukan login tanpa mengisi field mandatory</t>
+          <t>Melakukan login tanpa mengisi field username dan password</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -661,7 +661,7 @@
           <t>1. Berhasil membuka halaman login OrangeHRM.
 2. Field Username tetap kosong.
 3. Field Password tetap kosong.
-4. Berhasil menampilkan pesan validasi field mandatory.</t>
+4. Berhasil menampilkan pesan validasi field username dan password.</t>
         </is>
       </c>
     </row>
@@ -1385,7 +1385,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Melakukan login tanpa mengisi field mandatory</t>
+          <t>Melakukan login tanpa mengisi field username dan password</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -1411,7 +1411,7 @@
           <t>1. Berhasil membuka halaman login OrangeHRM.
 2. Field Username tetap kosong.
 3. Field Password tetap kosong.
-4. Berhasil menampilkan pesan validasi field mandatory.</t>
+4. Berhasil menampilkan pesan validasi field username dan password.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: implementasi bulk delete user (TC-ADMIN-11) dan sinkronisasi excel test case
</commit_message>
<xml_diff>
--- a/testcase/tc_orangehrm.xlsx
+++ b/testcase/tc_orangehrm.xlsx
@@ -13,9 +13,9 @@
     <sheet name="PIM" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gabungan'!$A$1:$G$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Gabungan'!$A$1:$G$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Authentication'!$A$1:$G$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Admin - User Management'!$A$1:$G$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Admin - User Management'!$A$1:$G$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'PIM'!$A$1:$G$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1106,37 +1106,80 @@
     <row r="17" ht="60" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>User Management</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Menghapus data System Users secara massal (Bulk Delete)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>1. Membuka halaman System Users.
+2. Mencentang beberapa checkbox data user.
+3. Klik button Delete Selected.
+4. Klik button Yes, Delete pada popup konfirmasi.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>1. Berhasil membuka halaman System Users.
+2. Berhasil memilih beberapa data user sekaligus.
+3. Berhasil menampilkan popup konfirmasi hapus.
+4. Berhasil menghapus seluruh data user terpilih secara massal dari daftar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="60" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>PIM</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Add Employee</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Menambahkan data Employee</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>1. Klik button Add.
 2. Mengisi semua field mandatory.
 3. Klik button Save.</t>
         </is>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>1. Berhasil membuka form Add Employee.
 2. Berhasil mengisi semua field mandatory.
@@ -1144,40 +1187,40 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="60" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="19" ht="60" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>PIM</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Add Employee</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Menambahkan data Employee tanpa mengisi field mandatory</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>Negative Case</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>1. Klik button Add.
 2. Mengosongkan field mandatory.
 3. Klik button Save.</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>1. Berhasil membuka form Add Employee.
 2. Field mandatory dibiarkan kosong.
@@ -1185,33 +1228,33 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="60" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20" ht="60" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>PIM</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Add Employee</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
         <is>
           <t>Menambahkan data Employee dengan upload foto profil</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>1. Klik button Add.
 2. Upload foto profil.
@@ -1219,7 +1262,7 @@
 4. Klik button Save.</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>1. Berhasil membuka form Add Employee.
 2. Berhasil mengupload foto profil.
@@ -1228,33 +1271,33 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="60" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="21" ht="60" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>PIM</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Add Employee</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Menambahkan data Employee dengan membuat login details</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>1. Klik button Add.
 2. Mengisi semua field mandatory.
@@ -1263,7 +1306,7 @@
 5. Klik button Save.</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>1. Berhasil membuka form Add Employee.
 2. Berhasil mengisi semua field mandatory.
@@ -1273,157 +1316,157 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="60" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="22" ht="60" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>PIM</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Employee List</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Mencari data Employee berdasarkan Employee Name</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>1. Mengisi field Employee Name dengan keyword valid.
 2. Klik button Search.</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>1. Berhasil mengisi field Employee Name.
 2. Berhasil menampilkan daftar data Employee sesuai keyword yang dimasukkan.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="60" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="23" ht="60" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>PIM</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>Employee List</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>Mencari data Employee berdasarkan Employee Id</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>1. Mengisi field Employee Id dengan keyword valid.
 2. Klik button Search.</t>
         </is>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>1. Berhasil mengisi field Employee Id.
 2. Berhasil menampilkan daftar data Employee sesuai keyword yang dimasukkan.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="60" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>PIM</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Employee List</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>Mereset filter Employee</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>1. Mengisi field filter yang tersedia.
 2. Klik button Reset.</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>1. Berhasil mengisi field filter.
 2. Berhasil mereset semua field filter ke kondisi awal dan menampilkan seluruh data Employee.</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="60" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="25" ht="60" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>PIM</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>Employee List</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>Mengubah data Employee</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>1. Klik icon Edit pada salah satu data Employee.
 2. Mengubah data pada field yang tersedia.
 3. Klik button Save.</t>
         </is>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>1. Berhasil membuka form Edit Employee.
 2. Berhasil mengubah data pada field yang dipilih.
@@ -1431,39 +1474,39 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="60" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="26" ht="60" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>PIM</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Employee List</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Menghapus data Employee</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>Positive Case</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>1. Klik icon Delete pada salah satu data Employee.
 2. Klik button Yes pada popup konfirmasi.</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>1. Berhasil menampilkan popup konfirmasi hapus.
 2. Berhasil menghapus data Employee dari daftar.</t>
@@ -1471,7 +1514,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G25"/>
+  <autoFilter ref="A1:G26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1754,7 +1797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2199,8 +2242,51 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>User Management</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Menghapus data System Users secara massal (Bulk Delete)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Positive Case</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>1. Membuka halaman System Users.
+2. Mencentang beberapa checkbox data user.
+3. Klik button Delete Selected.
+4. Klik button Yes, Delete pada popup konfirmasi.</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>1. Berhasil membuka halaman System Users.
+2. Berhasil memilih beberapa data user sekaligus.
+3. Berhasil menampilkan popup konfirmasi hapus.
+4. Berhasil menghapus seluruh data user terpilih secara massal dari daftar.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G11"/>
+  <autoFilter ref="A1:G12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>